<commit_message>
Update Synthetic Data for Week 3 and add new directory for Week 7 analysis
</commit_message>
<xml_diff>
--- a/week_3/SyntheticData.xlsx
+++ b/week_3/SyntheticData.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" firstSheet="2" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7450" firstSheet="2" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="17" r:id="rId1"/>
@@ -27,7 +27,7 @@
   </externalReferences>
   <calcPr calcId="152511"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId11"/>
+    <pivotCache cacheId="0" r:id="rId11"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1137,7 +1137,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1280,7 +1280,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1486,6 +1485,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1627,11 +1627,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="301426752"/>
-        <c:axId val="301419304"/>
+        <c:axId val="273256992"/>
+        <c:axId val="312360424"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="301426752"/>
+        <c:axId val="273256992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1663,6 +1663,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1697,7 +1698,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="301419304"/>
+        <c:crossAx val="312360424"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1705,7 +1706,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="301419304"/>
+        <c:axId val="312360424"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1746,6 +1747,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1780,7 +1782,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="301426752"/>
+        <c:crossAx val="273256992"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2194,11 +2196,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="301425184"/>
-        <c:axId val="301423224"/>
+        <c:axId val="273000688"/>
+        <c:axId val="312372296"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="301425184"/>
+        <c:axId val="273000688"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2264,7 +2266,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="301423224"/>
+        <c:crossAx val="312372296"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2272,7 +2274,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="301423224"/>
+        <c:axId val="312372296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2347,7 +2349,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="301425184"/>
+        <c:crossAx val="273000688"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3550,7 +3552,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -3753,7 +3755,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:O64" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:O62" totalsRowShown="0">
   <tableColumns count="15">
     <tableColumn id="1" name="loan_id" dataDxfId="12"/>
     <tableColumn id="2" name="inst_no" dataDxfId="11"/>
@@ -7046,7 +7048,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O64"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9" style="2" customWidth="1"/>
@@ -7165,7 +7167,7 @@
         <v>Current</v>
       </c>
       <c r="O2" s="7">
-        <v>45969</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -7216,11 +7218,11 @@
         <v>0</v>
       </c>
       <c r="N3" t="str">
-        <f t="shared" ref="N3:N64" si="1">IF(M3="","Current",IF(M3&lt;=0,"Current",IF(M3&lt;=7,"1–7",IF(M3&lt;=30,"8–30",IF(M3&lt;=60,"31–60",IF(M3&lt;=90,"61–90","90+"))))))</f>
+        <f t="shared" ref="N3:N62" si="1">IF(M3="","Current",IF(M3&lt;=0,"Current",IF(M3&lt;=7,"1–7",IF(M3&lt;=30,"8–30",IF(M3&lt;=60,"31–60",IF(M3&lt;=90,"61–90","90+"))))))</f>
         <v>Current</v>
       </c>
       <c r="O3" s="7">
-        <v>45970</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -7275,7 +7277,7 @@
         <v>Current</v>
       </c>
       <c r="O4" s="7">
-        <v>45971</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -7330,7 +7332,7 @@
         <v>Current</v>
       </c>
       <c r="O5" s="7">
-        <v>45972</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -7385,7 +7387,7 @@
         <v>Current</v>
       </c>
       <c r="O6" s="7">
-        <v>45973</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -7440,7 +7442,7 @@
         <v>Current</v>
       </c>
       <c r="O7" s="7">
-        <v>45974</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -7491,7 +7493,7 @@
         <v>Current</v>
       </c>
       <c r="O8" s="7">
-        <v>45975</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -7542,7 +7544,7 @@
         <v>Current</v>
       </c>
       <c r="O9" s="7">
-        <v>45976</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -7593,7 +7595,7 @@
         <v>Current</v>
       </c>
       <c r="O10" s="7">
-        <v>45977</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -7644,7 +7646,7 @@
         <v>Current</v>
       </c>
       <c r="O11" s="7">
-        <v>46008</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -7687,7 +7689,7 @@
         <v>84133.333333333328</v>
       </c>
       <c r="M12" s="37">
-        <f>MAX(0,L65-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L63-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N12" t="str">
@@ -7695,7 +7697,7 @@
         <v>Current</v>
       </c>
       <c r="O12" s="7">
-        <v>45979</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -7738,7 +7740,7 @@
         <v>126200</v>
       </c>
       <c r="M13" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>52</v>
       </c>
       <c r="N13" t="str">
@@ -7746,7 +7748,7 @@
         <v>31–60</v>
       </c>
       <c r="O13" s="7">
-        <v>45980</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -7790,7 +7792,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="37">
-        <f>MAX(0,L67-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L65-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N14" t="str">
@@ -7798,7 +7800,7 @@
         <v>Current</v>
       </c>
       <c r="O14" s="7">
-        <v>45981</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -7842,7 +7844,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="37">
-        <f>MAX(0,L68-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N15" t="str">
@@ -7850,7 +7852,7 @@
         <v>Current</v>
       </c>
       <c r="O15" s="7">
-        <v>45982</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -7894,7 +7896,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="37">
-        <f>MAX(0,L69-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L67-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N16" t="str">
@@ -7902,7 +7904,7 @@
         <v>Current</v>
       </c>
       <c r="O16" s="7">
-        <v>45983</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -7945,7 +7947,7 @@
         <v>57666.666666666664</v>
       </c>
       <c r="M17" s="37">
-        <f>MAX(0,L70-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L68-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N17" t="str">
@@ -7953,7 +7955,7 @@
         <v>Current</v>
       </c>
       <c r="O17" s="7">
-        <v>45984</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -7997,7 +7999,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="37">
-        <f>MAX(0,L71-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L69-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N18" t="str">
@@ -8005,7 +8007,7 @@
         <v>Current</v>
       </c>
       <c r="O18" s="7">
-        <v>45985</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -8053,7 +8055,7 @@
         <v>Current</v>
       </c>
       <c r="O19" s="7">
-        <v>45986</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -8108,7 +8110,7 @@
         <v>Current</v>
       </c>
       <c r="O20" s="7">
-        <v>45987</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -8163,7 +8165,7 @@
         <v>Current</v>
       </c>
       <c r="O21" s="7">
-        <v>45988</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -8210,7 +8212,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="37">
-        <f>MAX(0,L65-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L63-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N22" t="str">
@@ -8218,7 +8220,7 @@
         <v>Current</v>
       </c>
       <c r="O22" s="7">
-        <v>45989</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -8262,7 +8264,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>170</v>
       </c>
       <c r="N23" t="str">
@@ -8314,7 +8316,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>139</v>
       </c>
       <c r="N24" t="str">
@@ -8322,7 +8324,7 @@
         <v>90+</v>
       </c>
       <c r="O24" s="7">
-        <v>45991</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -8366,7 +8368,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>109</v>
       </c>
       <c r="N25" t="str">
@@ -8374,7 +8376,7 @@
         <v>90+</v>
       </c>
       <c r="O25" s="7">
-        <v>45992</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -8417,7 +8419,7 @@
         <v>18533.333333333332</v>
       </c>
       <c r="M26" s="37">
-        <f>MAX(0,L69-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L67-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N26" t="str">
@@ -8425,7 +8427,7 @@
         <v>Current</v>
       </c>
       <c r="O26" s="7">
-        <v>45993</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -8466,7 +8468,7 @@
       </c>
       <c r="K27" s="10"/>
       <c r="M27" s="37">
-        <f>MAX(0,L70-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L68-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N27" t="str">
@@ -8474,7 +8476,7 @@
         <v>Current</v>
       </c>
       <c r="O27" s="7">
-        <v>45994</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -8515,7 +8517,7 @@
       </c>
       <c r="K28" s="10"/>
       <c r="M28" s="37">
-        <f>MAX(0,L71-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L69-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N28" t="str">
@@ -8523,7 +8525,7 @@
         <v>Current</v>
       </c>
       <c r="O28" s="7">
-        <v>45995</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="29" spans="1:15">
@@ -8566,7 +8568,7 @@
         <v>38333.333333333336</v>
       </c>
       <c r="M29" s="37">
-        <f>MAX(0,L72-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L70-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N29" t="str">
@@ -8574,7 +8576,7 @@
         <v>Current</v>
       </c>
       <c r="O29" s="7">
-        <v>45996</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -8617,7 +8619,7 @@
         <v>76666.666666666672</v>
       </c>
       <c r="M30" s="37">
-        <f>MAX(0,L73-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L71-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N30" t="str">
@@ -8625,7 +8627,7 @@
         <v>Current</v>
       </c>
       <c r="O30" s="7">
-        <v>45997</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="31" spans="1:15">
@@ -8668,7 +8670,7 @@
         <v>115000</v>
       </c>
       <c r="M31" s="37">
-        <f>MAX(0,L74-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L72-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N31" t="str">
@@ -8676,7 +8678,7 @@
         <v>Current</v>
       </c>
       <c r="O31" s="7">
-        <v>45998</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -8720,7 +8722,7 @@
         <v>0</v>
       </c>
       <c r="M32" s="37">
-        <f>MAX(0,L75-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L73-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N32" t="str">
@@ -8728,7 +8730,7 @@
         <v>Current</v>
       </c>
       <c r="O32" s="7">
-        <v>45999</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="33" spans="1:15">
@@ -8772,7 +8774,7 @@
         <v>0</v>
       </c>
       <c r="M33" s="37">
-        <f>MAX(0,L76-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L74-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N33" t="str">
@@ -8780,7 +8782,7 @@
         <v>Current</v>
       </c>
       <c r="O33" s="7">
-        <v>46000</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="34" spans="1:15">
@@ -8824,7 +8826,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="37">
-        <f>MAX(0,L77-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L75-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N34" t="str">
@@ -8832,7 +8834,7 @@
         <v>Current</v>
       </c>
       <c r="O34" s="7">
-        <v>46001</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="35" spans="1:15">
@@ -8875,7 +8877,7 @@
         <v>53266.666666666664</v>
       </c>
       <c r="M35" s="37">
-        <f>MAX(0,L78-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L76-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N35" t="str">
@@ -8883,7 +8885,7 @@
         <v>Current</v>
       </c>
       <c r="O35" s="7">
-        <v>46002</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="36" spans="1:15">
@@ -8927,7 +8929,7 @@
         <v>0</v>
       </c>
       <c r="M36" s="37">
-        <f>MAX(0,L79-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L77-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N36" t="str">
@@ -8935,7 +8937,7 @@
         <v>Current</v>
       </c>
       <c r="O36" s="7">
-        <v>46003</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="37" spans="1:15">
@@ -8979,7 +8981,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="37">
-        <f>MAX(0,L80-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L78-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N37" t="str">
@@ -8987,7 +8989,7 @@
         <v>Current</v>
       </c>
       <c r="O37" s="7">
-        <v>46004</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="38" spans="1:15">
@@ -9034,7 +9036,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="37">
-        <f>MAX(0,L81-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L79-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N38" t="str">
@@ -9042,7 +9044,7 @@
         <v>Current</v>
       </c>
       <c r="O38" s="7">
-        <v>46005</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="39" spans="1:15">
@@ -9089,7 +9091,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="37">
-        <f>MAX(0,L82-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L80-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N39" t="str">
@@ -9097,7 +9099,7 @@
         <v>Current</v>
       </c>
       <c r="O39" s="7">
-        <v>46006</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="40" spans="1:15">
@@ -9144,7 +9146,7 @@
         <v>0</v>
       </c>
       <c r="M40" s="37">
-        <f>MAX(0,L83-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L81-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N40" t="str">
@@ -9152,7 +9154,7 @@
         <v>Current</v>
       </c>
       <c r="O40" s="7">
-        <v>46007</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="41" spans="1:15">
@@ -9196,7 +9198,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>164</v>
       </c>
       <c r="N41" t="str">
@@ -9204,7 +9206,7 @@
         <v>90+</v>
       </c>
       <c r="O41" s="7">
-        <v>46008</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="42" spans="1:15">
@@ -9248,7 +9250,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>133</v>
       </c>
       <c r="N42" t="str">
@@ -9256,7 +9258,7 @@
         <v>90+</v>
       </c>
       <c r="O42" s="7">
-        <v>46009</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="43" spans="1:15">
@@ -9300,7 +9302,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>103</v>
       </c>
       <c r="N43" t="str">
@@ -9308,7 +9310,7 @@
         <v>90+</v>
       </c>
       <c r="O43" s="7">
-        <v>46010</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="44" spans="1:15">
@@ -9339,7 +9341,7 @@
       <c r="J44" s="12"/>
       <c r="K44" s="10"/>
       <c r="M44" s="37">
-        <f>MAX(0,L87-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L85-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N44" t="str">
@@ -9347,7 +9349,7 @@
         <v>Current</v>
       </c>
       <c r="O44" s="7">
-        <v>46011</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="45" spans="1:15">
@@ -9378,7 +9380,7 @@
       <c r="J45" s="12"/>
       <c r="K45" s="10"/>
       <c r="M45" s="37">
-        <f>MAX(0,L88-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L86-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N45" t="str">
@@ -9386,7 +9388,7 @@
         <v>Current</v>
       </c>
       <c r="O45" s="7">
-        <v>46012</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="46" spans="1:15">
@@ -9417,7 +9419,7 @@
       <c r="J46" s="12"/>
       <c r="K46" s="10"/>
       <c r="M46" s="37">
-        <f>MAX(0,L89-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L87-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N46" t="str">
@@ -9425,7 +9427,7 @@
         <v>Current</v>
       </c>
       <c r="O46" s="7">
-        <v>46013</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="47" spans="1:15">
@@ -9456,7 +9458,7 @@
       <c r="J47" s="12"/>
       <c r="K47" s="12"/>
       <c r="M47" s="37">
-        <f>MAX(0,L90-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L88-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N47" t="str">
@@ -9464,7 +9466,7 @@
         <v>Current</v>
       </c>
       <c r="O47" s="7">
-        <v>46014</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="48" spans="1:15">
@@ -9495,7 +9497,7 @@
       <c r="J48" s="12"/>
       <c r="K48" s="12"/>
       <c r="M48" s="37">
-        <f>MAX(0,L91-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L89-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N48" t="str">
@@ -9503,7 +9505,7 @@
         <v>Current</v>
       </c>
       <c r="O48" s="7">
-        <v>46015</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="49" spans="1:15">
@@ -9534,7 +9536,7 @@
       <c r="J49" s="12"/>
       <c r="K49" s="12"/>
       <c r="M49" s="37">
-        <f>MAX(0,L92-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L90-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N49" t="str">
@@ -9542,7 +9544,7 @@
         <v>Current</v>
       </c>
       <c r="O49" s="7">
-        <v>46016</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="50" spans="1:15">
@@ -9586,7 +9588,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="37">
-        <f>MAX(0,L93-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L91-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N50" t="str">
@@ -9594,7 +9596,7 @@
         <v>Current</v>
       </c>
       <c r="O50" s="7">
-        <v>46017</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="51" spans="1:15">
@@ -9638,7 +9640,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="37">
-        <f>MAX(0,L94-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L92-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N51" t="str">
@@ -9646,7 +9648,7 @@
         <v>Current</v>
       </c>
       <c r="O51" s="7">
-        <v>46018</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="52" spans="1:15">
@@ -9690,7 +9692,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="37">
-        <f>MAX(0,L95-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L93-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N52" t="str">
@@ -9698,7 +9700,7 @@
         <v>Current</v>
       </c>
       <c r="O52" s="7">
-        <v>46019</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="53" spans="1:15">
@@ -9729,7 +9731,7 @@
       <c r="J53" s="12"/>
       <c r="K53" s="10"/>
       <c r="M53" s="37">
-        <f>MAX(0,L96-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L94-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N53" t="str">
@@ -9737,7 +9739,7 @@
         <v>Current</v>
       </c>
       <c r="O53" s="7">
-        <v>46020</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="54" spans="1:15">
@@ -9768,7 +9770,7 @@
       <c r="J54" s="12"/>
       <c r="K54" s="10"/>
       <c r="M54" s="37">
-        <f>MAX(0,L97-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L95-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N54" t="str">
@@ -9776,7 +9778,7 @@
         <v>Current</v>
       </c>
       <c r="O54" s="7">
-        <v>46021</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="55" spans="1:15">
@@ -9807,7 +9809,7 @@
       <c r="J55" s="12"/>
       <c r="K55" s="10"/>
       <c r="M55" s="37">
-        <f>MAX(0,L98-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L96-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N55" t="str">
@@ -9815,7 +9817,7 @@
         <v>Current</v>
       </c>
       <c r="O55" s="7">
-        <v>46022</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="56" spans="1:15">
@@ -9862,7 +9864,7 @@
         <v>0</v>
       </c>
       <c r="M56" s="37">
-        <f>MAX(0,L99-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L97-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N56" t="str">
@@ -9870,7 +9872,7 @@
         <v>Current</v>
       </c>
       <c r="O56" s="7">
-        <v>46023</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="57" spans="1:15">
@@ -9917,7 +9919,7 @@
         <v>0</v>
       </c>
       <c r="M57" s="37">
-        <f>MAX(0,L100-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L98-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N57" t="str">
@@ -9925,7 +9927,7 @@
         <v>Current</v>
       </c>
       <c r="O57" s="7">
-        <v>46024</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="58" spans="1:15">
@@ -9972,7 +9974,7 @@
         <v>0</v>
       </c>
       <c r="M58" s="37">
-        <f>MAX(0,L101-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L99-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N58" t="str">
@@ -9980,7 +9982,7 @@
         <v>Current</v>
       </c>
       <c r="O58" s="7">
-        <v>46025</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="59" spans="1:15">
@@ -10020,7 +10022,7 @@
         <v>0</v>
       </c>
       <c r="M59" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>158</v>
       </c>
       <c r="N59" t="str">
@@ -10028,7 +10030,7 @@
         <v>90+</v>
       </c>
       <c r="O59" s="7">
-        <v>46026</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="60" spans="1:15">
@@ -10068,7 +10070,7 @@
         <v>0</v>
       </c>
       <c r="M60" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>127</v>
       </c>
       <c r="N60" t="str">
@@ -10076,7 +10078,7 @@
         <v>90+</v>
       </c>
       <c r="O60" s="7">
-        <v>46027</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="61" spans="1:15">
@@ -10116,7 +10118,7 @@
         <v>0</v>
       </c>
       <c r="M61" s="37">
-        <f>MAX(0,L66-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L64-Table1[[#This Row],[due_date]])</f>
         <v>97</v>
       </c>
       <c r="N61" t="str">
@@ -10124,7 +10126,7 @@
         <v>90+</v>
       </c>
       <c r="O61" s="7">
-        <v>46028</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="62" spans="1:15">
@@ -10137,7 +10139,7 @@
       <c r="J62" s="12"/>
       <c r="K62" s="10"/>
       <c r="M62" s="37">
-        <f>MAX(0,L105-Table1[[#This Row],[due_date]])</f>
+        <f>MAX(0,L103-Table1[[#This Row],[due_date]])</f>
         <v>0</v>
       </c>
       <c r="N62" t="str">
@@ -10145,56 +10147,14 @@
         <v>Current</v>
       </c>
       <c r="O62" s="7">
-        <v>46029</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="19"/>
-      <c r="E63" s="19"/>
-      <c r="G63" s="12"/>
-      <c r="J63" s="12"/>
-      <c r="K63" s="10"/>
-      <c r="M63" s="37">
-        <f>MAX(0,L104-Table1[[#This Row],[due_date]])</f>
-        <v>0</v>
-      </c>
-      <c r="N63" t="str">
-        <f t="shared" si="1"/>
-        <v>Current</v>
-      </c>
-      <c r="O63" s="78">
-        <f>L123</f>
-        <v>0</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="64" spans="1:15">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="19"/>
-      <c r="E64" s="19"/>
-      <c r="G64" s="12"/>
-      <c r="J64" s="12"/>
-      <c r="K64" s="10"/>
-      <c r="M64" s="37">
-        <f>MAX(0,L105-Table1[[#This Row],[due_date]])</f>
-        <v>0</v>
-      </c>
-      <c r="N64" t="str">
-        <f t="shared" si="1"/>
-        <v>Current</v>
-      </c>
-      <c r="O64" s="78">
-        <f>L124</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="11:12">
-      <c r="K66" s="2" t="s">
+      <c r="K64" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="L66" s="7">
+      <c r="L64" s="7">
         <v>46050</v>
       </c>
     </row>
@@ -10662,67 +10622,67 @@
       <c r="B6" s="52" t="s">
         <v>188</v>
       </c>
-      <c r="C6" s="85">
+      <c r="C6" s="84">
         <v>46050</v>
       </c>
-      <c r="D6" s="85"/>
-      <c r="F6" s="86" t="s">
+      <c r="D6" s="84"/>
+      <c r="F6" s="85" t="s">
         <v>246</v>
       </c>
-      <c r="G6" s="86"/>
-      <c r="H6" s="86"/>
-      <c r="I6" s="86"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="85"/>
+      <c r="K6" s="85"/>
+      <c r="L6" s="85"/>
     </row>
     <row r="7" spans="2:21" ht="15" customHeight="1">
       <c r="B7" s="52" t="s">
         <v>229</v>
       </c>
-      <c r="C7" s="87" t="s">
+      <c r="C7" s="86" t="s">
         <v>247</v>
       </c>
-      <c r="D7" s="87"/>
-      <c r="F7" s="86"/>
-      <c r="G7" s="86"/>
-      <c r="H7" s="86"/>
-      <c r="I7" s="86"/>
-      <c r="J7" s="86"/>
-      <c r="K7" s="86"/>
-      <c r="L7" s="86"/>
+      <c r="D7" s="86"/>
+      <c r="F7" s="85"/>
+      <c r="G7" s="85"/>
+      <c r="H7" s="85"/>
+      <c r="I7" s="85"/>
+      <c r="J7" s="85"/>
+      <c r="K7" s="85"/>
+      <c r="L7" s="85"/>
     </row>
     <row r="8" spans="2:21" ht="15" customHeight="1">
       <c r="B8" s="52" t="s">
         <v>226</v>
       </c>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="86" t="s">
         <v>247</v>
       </c>
-      <c r="D8" s="87"/>
-      <c r="F8" s="86"/>
-      <c r="G8" s="86"/>
-      <c r="H8" s="86"/>
-      <c r="I8" s="86"/>
-      <c r="J8" s="86"/>
-      <c r="K8" s="86"/>
-      <c r="L8" s="86"/>
+      <c r="D8" s="86"/>
+      <c r="F8" s="85"/>
+      <c r="G8" s="85"/>
+      <c r="H8" s="85"/>
+      <c r="I8" s="85"/>
+      <c r="J8" s="85"/>
+      <c r="K8" s="85"/>
+      <c r="L8" s="85"/>
     </row>
     <row r="9" spans="2:21" ht="15" customHeight="1">
       <c r="B9" s="52" t="s">
         <v>223</v>
       </c>
-      <c r="C9" s="87" t="s">
+      <c r="C9" s="86" t="s">
         <v>247</v>
       </c>
-      <c r="D9" s="87"/>
-      <c r="F9" s="86"/>
-      <c r="G9" s="86"/>
-      <c r="H9" s="86"/>
-      <c r="I9" s="86"/>
-      <c r="J9" s="86"/>
-      <c r="K9" s="86"/>
-      <c r="L9" s="86"/>
+      <c r="D9" s="86"/>
+      <c r="F9" s="85"/>
+      <c r="G9" s="85"/>
+      <c r="H9" s="85"/>
+      <c r="I9" s="85"/>
+      <c r="J9" s="85"/>
+      <c r="K9" s="85"/>
+      <c r="L9" s="85"/>
     </row>
     <row r="11" spans="2:21" ht="15" customHeight="1">
       <c r="B11" s="51" t="s">
@@ -10736,113 +10696,113 @@
       </c>
     </row>
     <row r="13" spans="2:21" ht="15" customHeight="1">
-      <c r="B13" s="81" t="s">
+      <c r="B13" s="80" t="s">
         <v>191</v>
       </c>
-      <c r="C13" s="81"/>
-      <c r="D13" s="81"/>
-      <c r="E13" s="81" t="s">
+      <c r="C13" s="80"/>
+      <c r="D13" s="80"/>
+      <c r="E13" s="80" t="s">
         <v>194</v>
       </c>
-      <c r="F13" s="81"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="81" t="s">
+      <c r="F13" s="80"/>
+      <c r="G13" s="80"/>
+      <c r="H13" s="80" t="s">
         <v>197</v>
       </c>
-      <c r="I13" s="81"/>
-      <c r="J13" s="81"/>
-      <c r="K13" s="81" t="s">
+      <c r="I13" s="80"/>
+      <c r="J13" s="80"/>
+      <c r="K13" s="80" t="s">
         <v>200</v>
       </c>
-      <c r="L13" s="81"/>
-      <c r="M13" s="81"/>
-      <c r="N13" s="81" t="s">
+      <c r="L13" s="80"/>
+      <c r="M13" s="80"/>
+      <c r="N13" s="80" t="s">
         <v>203</v>
       </c>
-      <c r="O13" s="81"/>
-      <c r="P13" s="81"/>
-      <c r="Q13" s="81" t="s">
+      <c r="O13" s="80"/>
+      <c r="P13" s="80"/>
+      <c r="Q13" s="80" t="s">
         <v>206</v>
       </c>
-      <c r="R13" s="81"/>
-      <c r="S13" s="81"/>
+      <c r="R13" s="80"/>
+      <c r="S13" s="80"/>
     </row>
     <row r="14" spans="2:21" ht="15" customHeight="1">
-      <c r="B14" s="82">
+      <c r="B14" s="81">
         <v>20</v>
       </c>
-      <c r="C14" s="82"/>
-      <c r="D14" s="82"/>
-      <c r="E14" s="82">
+      <c r="C14" s="81"/>
+      <c r="D14" s="81"/>
+      <c r="E14" s="81">
         <f>SUMPRODUCT(('[1]Calc - Loan Summary'!$J$5:$J$24=1)*('[1]Calc - Loan Summary'!$O$5:$O$24&gt;0)*(('[1]Calc - Loan Summary'!$C$5:$C$24=$C$7)+($C$7="All")&gt;0)*(('[1]Calc - Loan Summary'!$D$5:$D$24=$C$8)+($C$8="All")&gt;0)*(('[1]Calc - Loan Summary'!$E$5:$E$24=$C$9)+($C$9="All")&gt;0))</f>
         <v>13</v>
       </c>
-      <c r="F14" s="82"/>
-      <c r="G14" s="82"/>
-      <c r="H14" s="83">
+      <c r="F14" s="81"/>
+      <c r="G14" s="81"/>
+      <c r="H14" s="82">
         <f>SUM(Installment!H8:H61)</f>
         <v>431666.66666666657</v>
       </c>
-      <c r="I14" s="83"/>
-      <c r="J14" s="83"/>
-      <c r="K14" s="83">
+      <c r="I14" s="82"/>
+      <c r="J14" s="82"/>
+      <c r="K14" s="82">
         <f>SUM(Installment!D2:D61)</f>
         <v>2520299.9999999995</v>
       </c>
-      <c r="L14" s="83"/>
-      <c r="M14" s="83"/>
-      <c r="N14" s="83">
+      <c r="L14" s="82"/>
+      <c r="M14" s="82"/>
+      <c r="N14" s="82">
         <f>SUM(Installment!J2:J61)</f>
         <v>3416466.666666667</v>
       </c>
-      <c r="O14" s="83"/>
-      <c r="P14" s="83"/>
-      <c r="Q14" s="84">
+      <c r="O14" s="82"/>
+      <c r="P14" s="82"/>
+      <c r="Q14" s="83">
         <f>IFERROR(N14/K14,0)</f>
         <v>1.3555793622452357</v>
       </c>
-      <c r="R14" s="84"/>
-      <c r="S14" s="84"/>
+      <c r="R14" s="83"/>
+      <c r="S14" s="83"/>
     </row>
     <row r="15" spans="2:21" ht="15" customHeight="1">
-      <c r="B15" s="82"/>
-      <c r="C15" s="82"/>
-      <c r="D15" s="82"/>
-      <c r="E15" s="82"/>
-      <c r="F15" s="82"/>
-      <c r="G15" s="82"/>
-      <c r="H15" s="83"/>
-      <c r="I15" s="83"/>
-      <c r="J15" s="83"/>
-      <c r="K15" s="83"/>
-      <c r="L15" s="83"/>
-      <c r="M15" s="83"/>
-      <c r="N15" s="83"/>
-      <c r="O15" s="83"/>
-      <c r="P15" s="83"/>
-      <c r="Q15" s="84"/>
-      <c r="R15" s="84"/>
-      <c r="S15" s="84"/>
+      <c r="B15" s="81"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="81"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="81"/>
+      <c r="H15" s="82"/>
+      <c r="I15" s="82"/>
+      <c r="J15" s="82"/>
+      <c r="K15" s="82"/>
+      <c r="L15" s="82"/>
+      <c r="M15" s="82"/>
+      <c r="N15" s="82"/>
+      <c r="O15" s="82"/>
+      <c r="P15" s="82"/>
+      <c r="Q15" s="83"/>
+      <c r="R15" s="83"/>
+      <c r="S15" s="83"/>
     </row>
     <row r="16" spans="2:21" ht="15" customHeight="1">
-      <c r="B16" s="82"/>
-      <c r="C16" s="82"/>
-      <c r="D16" s="82"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="82"/>
-      <c r="G16" s="82"/>
-      <c r="H16" s="83"/>
-      <c r="I16" s="83"/>
-      <c r="J16" s="83"/>
-      <c r="K16" s="83"/>
-      <c r="L16" s="83"/>
-      <c r="M16" s="83"/>
-      <c r="N16" s="83"/>
-      <c r="O16" s="83"/>
-      <c r="P16" s="83"/>
-      <c r="Q16" s="84"/>
-      <c r="R16" s="84"/>
-      <c r="S16" s="84"/>
+      <c r="B16" s="81"/>
+      <c r="C16" s="81"/>
+      <c r="D16" s="81"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="81"/>
+      <c r="G16" s="81"/>
+      <c r="H16" s="82"/>
+      <c r="I16" s="82"/>
+      <c r="J16" s="82"/>
+      <c r="K16" s="82"/>
+      <c r="L16" s="82"/>
+      <c r="M16" s="82"/>
+      <c r="N16" s="82"/>
+      <c r="O16" s="82"/>
+      <c r="P16" s="82"/>
+      <c r="Q16" s="83"/>
+      <c r="R16" s="83"/>
+      <c r="S16" s="83"/>
     </row>
     <row r="18" spans="2:7" ht="15" customHeight="1">
       <c r="B18" s="51" t="s">
@@ -11182,159 +11142,159 @@
       </c>
     </row>
     <row r="38" spans="2:15" ht="18" customHeight="1">
-      <c r="B38" s="80" t="s">
+      <c r="B38" s="79" t="s">
         <v>269</v>
       </c>
-      <c r="C38" s="80"/>
-      <c r="D38" s="80"/>
-      <c r="E38" s="80"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="80"/>
-      <c r="H38" s="80"/>
-      <c r="I38" s="80"/>
-      <c r="J38" s="80"/>
-      <c r="K38" s="80"/>
-      <c r="L38" s="80"/>
-      <c r="M38" s="80"/>
-      <c r="N38" s="80"/>
-      <c r="O38" s="80"/>
+      <c r="C38" s="79"/>
+      <c r="D38" s="79"/>
+      <c r="E38" s="79"/>
+      <c r="F38" s="79"/>
+      <c r="G38" s="79"/>
+      <c r="H38" s="79"/>
+      <c r="I38" s="79"/>
+      <c r="J38" s="79"/>
+      <c r="K38" s="79"/>
+      <c r="L38" s="79"/>
+      <c r="M38" s="79"/>
+      <c r="N38" s="79"/>
+      <c r="O38" s="79"/>
     </row>
     <row r="39" spans="2:15" ht="84.75" customHeight="1">
-      <c r="B39" s="79" t="s">
+      <c r="B39" s="78" t="s">
         <v>270</v>
       </c>
-      <c r="C39" s="79"/>
-      <c r="D39" s="79"/>
-      <c r="E39" s="79"/>
-      <c r="F39" s="79"/>
-      <c r="G39" s="79"/>
-      <c r="H39" s="79"/>
-      <c r="I39" s="79"/>
-      <c r="J39" s="79"/>
-      <c r="K39" s="79"/>
-      <c r="L39" s="79"/>
-      <c r="M39" s="79"/>
-      <c r="N39" s="79"/>
-      <c r="O39" s="79"/>
+      <c r="C39" s="78"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
+      <c r="F39" s="78"/>
+      <c r="G39" s="78"/>
+      <c r="H39" s="78"/>
+      <c r="I39" s="78"/>
+      <c r="J39" s="78"/>
+      <c r="K39" s="78"/>
+      <c r="L39" s="78"/>
+      <c r="M39" s="78"/>
+      <c r="N39" s="78"/>
+      <c r="O39" s="78"/>
     </row>
     <row r="40" spans="2:15" ht="18" customHeight="1">
       <c r="B40" s="67" t="s">
         <v>271</v>
       </c>
-      <c r="C40" s="79" t="s">
+      <c r="C40" s="78" t="s">
         <v>272</v>
       </c>
-      <c r="D40" s="79"/>
-      <c r="E40" s="79"/>
-      <c r="F40" s="79"/>
-      <c r="G40" s="79"/>
-      <c r="H40" s="79"/>
-      <c r="I40" s="79"/>
-      <c r="J40" s="79"/>
-      <c r="K40" s="79"/>
-      <c r="L40" s="79"/>
-      <c r="M40" s="79"/>
-      <c r="N40" s="79"/>
-      <c r="O40" s="79"/>
+      <c r="D40" s="78"/>
+      <c r="E40" s="78"/>
+      <c r="F40" s="78"/>
+      <c r="G40" s="78"/>
+      <c r="H40" s="78"/>
+      <c r="I40" s="78"/>
+      <c r="J40" s="78"/>
+      <c r="K40" s="78"/>
+      <c r="L40" s="78"/>
+      <c r="M40" s="78"/>
+      <c r="N40" s="78"/>
+      <c r="O40" s="78"/>
     </row>
     <row r="41" spans="2:15" ht="64.5" customHeight="1">
       <c r="B41" s="68" t="s">
         <v>273</v>
       </c>
-      <c r="C41" s="79" t="s">
+      <c r="C41" s="78" t="s">
         <v>274</v>
       </c>
-      <c r="D41" s="79"/>
-      <c r="E41" s="79"/>
-      <c r="F41" s="79"/>
-      <c r="G41" s="79"/>
-      <c r="H41" s="79"/>
-      <c r="I41" s="79"/>
-      <c r="J41" s="79"/>
-      <c r="K41" s="79"/>
-      <c r="L41" s="79"/>
-      <c r="M41" s="79"/>
-      <c r="N41" s="79"/>
-      <c r="O41" s="79"/>
+      <c r="D41" s="78"/>
+      <c r="E41" s="78"/>
+      <c r="F41" s="78"/>
+      <c r="G41" s="78"/>
+      <c r="H41" s="78"/>
+      <c r="I41" s="78"/>
+      <c r="J41" s="78"/>
+      <c r="K41" s="78"/>
+      <c r="L41" s="78"/>
+      <c r="M41" s="78"/>
+      <c r="N41" s="78"/>
+      <c r="O41" s="78"/>
     </row>
     <row r="42" spans="2:15" ht="45" customHeight="1">
       <c r="B42" s="69"/>
     </row>
     <row r="43" spans="2:15" ht="18" customHeight="1">
-      <c r="B43" s="80" t="s">
+      <c r="B43" s="79" t="s">
         <v>275</v>
       </c>
-      <c r="C43" s="80"/>
-      <c r="D43" s="80"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="80"/>
-      <c r="G43" s="80"/>
-      <c r="H43" s="80"/>
-      <c r="I43" s="80"/>
-      <c r="J43" s="80"/>
-      <c r="K43" s="80"/>
-      <c r="L43" s="80"/>
-      <c r="M43" s="80"/>
-      <c r="N43" s="80"/>
-      <c r="O43" s="80"/>
+      <c r="C43" s="79"/>
+      <c r="D43" s="79"/>
+      <c r="E43" s="79"/>
+      <c r="F43" s="79"/>
+      <c r="G43" s="79"/>
+      <c r="H43" s="79"/>
+      <c r="I43" s="79"/>
+      <c r="J43" s="79"/>
+      <c r="K43" s="79"/>
+      <c r="L43" s="79"/>
+      <c r="M43" s="79"/>
+      <c r="N43" s="79"/>
+      <c r="O43" s="79"/>
     </row>
     <row r="44" spans="2:15" ht="69.75" customHeight="1">
-      <c r="B44" s="79" t="s">
+      <c r="B44" s="78" t="s">
         <v>276</v>
       </c>
-      <c r="C44" s="79"/>
-      <c r="D44" s="79"/>
-      <c r="E44" s="79"/>
-      <c r="F44" s="79"/>
-      <c r="G44" s="79"/>
-      <c r="H44" s="79"/>
-      <c r="I44" s="79"/>
-      <c r="J44" s="79"/>
-      <c r="K44" s="79"/>
-      <c r="L44" s="79"/>
-      <c r="M44" s="79"/>
-      <c r="N44" s="79"/>
-      <c r="O44" s="79"/>
+      <c r="C44" s="78"/>
+      <c r="D44" s="78"/>
+      <c r="E44" s="78"/>
+      <c r="F44" s="78"/>
+      <c r="G44" s="78"/>
+      <c r="H44" s="78"/>
+      <c r="I44" s="78"/>
+      <c r="J44" s="78"/>
+      <c r="K44" s="78"/>
+      <c r="L44" s="78"/>
+      <c r="M44" s="78"/>
+      <c r="N44" s="78"/>
+      <c r="O44" s="78"/>
     </row>
     <row r="45" spans="2:15" ht="31.5" customHeight="1">
       <c r="B45" s="67" t="s">
         <v>271</v>
       </c>
-      <c r="C45" s="79" t="s">
+      <c r="C45" s="78" t="s">
         <v>277</v>
       </c>
-      <c r="D45" s="79"/>
-      <c r="E45" s="79"/>
-      <c r="F45" s="79"/>
-      <c r="G45" s="79"/>
-      <c r="H45" s="79"/>
-      <c r="I45" s="79"/>
-      <c r="J45" s="79"/>
-      <c r="K45" s="79"/>
-      <c r="L45" s="79"/>
-      <c r="M45" s="79"/>
-      <c r="N45" s="79"/>
-      <c r="O45" s="79"/>
+      <c r="D45" s="78"/>
+      <c r="E45" s="78"/>
+      <c r="F45" s="78"/>
+      <c r="G45" s="78"/>
+      <c r="H45" s="78"/>
+      <c r="I45" s="78"/>
+      <c r="J45" s="78"/>
+      <c r="K45" s="78"/>
+      <c r="L45" s="78"/>
+      <c r="M45" s="78"/>
+      <c r="N45" s="78"/>
+      <c r="O45" s="78"/>
     </row>
     <row r="46" spans="2:15" ht="54.75" customHeight="1">
       <c r="B46" s="67" t="s">
         <v>273</v>
       </c>
-      <c r="C46" s="79" t="s">
+      <c r="C46" s="78" t="s">
         <v>278</v>
       </c>
-      <c r="D46" s="79"/>
-      <c r="E46" s="79"/>
-      <c r="F46" s="79"/>
-      <c r="G46" s="79"/>
-      <c r="H46" s="79"/>
-      <c r="I46" s="79"/>
-      <c r="J46" s="79"/>
-      <c r="K46" s="79"/>
-      <c r="L46" s="79"/>
-      <c r="M46" s="79"/>
-      <c r="N46" s="79"/>
-      <c r="O46" s="79"/>
+      <c r="D46" s="78"/>
+      <c r="E46" s="78"/>
+      <c r="F46" s="78"/>
+      <c r="G46" s="78"/>
+      <c r="H46" s="78"/>
+      <c r="I46" s="78"/>
+      <c r="J46" s="78"/>
+      <c r="K46" s="78"/>
+      <c r="L46" s="78"/>
+      <c r="M46" s="78"/>
+      <c r="N46" s="78"/>
+      <c r="O46" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="25">

</xml_diff>